<commit_message>
Corrections to prior flight data for EOSS-391 to EOSS-403 to properly convert 'packettime' to the local timezone
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/eoss-392.xlsx
+++ b/www/flightdata/xlsx/eoss-392.xlsx
@@ -2580,7 +2580,7 @@
         <v>46116.28911207176</v>
       </c>
       <c r="D2" s="1">
-        <v>46116.53905092592</v>
+        <v>46116.28905092592</v>
       </c>
       <c r="E2">
         <v>5210</v>
@@ -2687,7 +2687,7 @@
         <v>46116.28909122685</v>
       </c>
       <c r="D3" s="1">
-        <v>46116.5390625</v>
+        <v>46116.2890625</v>
       </c>
       <c r="E3">
         <v>5272</v>
@@ -2818,7 +2818,7 @@
         <v>46116.28943557871</v>
       </c>
       <c r="D4" s="1">
-        <v>46116.53939814815</v>
+        <v>46116.28939814815</v>
       </c>
       <c r="E4">
         <v>5757</v>
@@ -2961,7 +2961,7 @@
         <v>46116.28943055555</v>
       </c>
       <c r="D5" s="1">
-        <v>46116.53940972222</v>
+        <v>46116.28940972222</v>
       </c>
       <c r="E5">
         <v>5847</v>
@@ -3104,7 +3104,7 @@
         <v>46116.289811076385</v>
       </c>
       <c r="D6" s="1">
-        <v>46116.53974537037</v>
+        <v>46116.28974537037</v>
       </c>
       <c r="E6">
         <v>6368</v>
@@ -3247,7 +3247,7 @@
         <v>46116.28977811342</v>
       </c>
       <c r="D7" s="1">
-        <v>46116.53975694445</v>
+        <v>46116.28975694445</v>
       </c>
       <c r="E7">
         <v>6460</v>
@@ -3390,7 +3390,7 @@
         <v>46116.29012508102</v>
       </c>
       <c r="D8" s="1">
-        <v>46116.54010416667</v>
+        <v>46116.29010416667</v>
       </c>
       <c r="E8">
         <v>7108</v>
@@ -3533,7 +3533,7 @@
         <v>46116.29050587963</v>
       </c>
       <c r="D9" s="1">
-        <v>46116.54043981482</v>
+        <v>46116.29043981482</v>
       </c>
       <c r="E9">
         <v>7639</v>
@@ -3676,7 +3676,7 @@
         <v>46116.290472002314</v>
       </c>
       <c r="D10" s="1">
-        <v>46116.540451388886</v>
+        <v>46116.290451388886</v>
       </c>
       <c r="E10">
         <v>7727</v>
@@ -3819,7 +3819,7 @@
         <v>46116.29081947917</v>
       </c>
       <c r="D11" s="1">
-        <v>46116.54079861111</v>
+        <v>46116.29079861111</v>
       </c>
       <c r="E11">
         <v>8388</v>
@@ -3962,7 +3962,7 @@
         <v>46116.29119988426</v>
       </c>
       <c r="D12" s="1">
-        <v>46116.541134259256</v>
+        <v>46116.291134259256</v>
       </c>
       <c r="E12">
         <v>8933</v>
@@ -4105,7 +4105,7 @@
         <v>46116.291167048614</v>
       </c>
       <c r="D13" s="1">
-        <v>46116.54114583333</v>
+        <v>46116.29114583333</v>
       </c>
       <c r="E13">
         <v>9047</v>
@@ -4248,7 +4248,7 @@
         <v>46116.291514282406</v>
       </c>
       <c r="D14" s="1">
-        <v>46116.541493055556</v>
+        <v>46116.291493055556</v>
       </c>
       <c r="E14">
         <v>9703</v>
@@ -4391,7 +4391,7 @@
         <v>46116.291894131944</v>
       </c>
       <c r="D15" s="1">
-        <v>46116.5418287037</v>
+        <v>46116.2918287037</v>
       </c>
       <c r="E15">
         <v>10303</v>
@@ -4534,7 +4534,7 @@
         <v>46116.291861516205</v>
       </c>
       <c r="D16" s="1">
-        <v>46116.54184027778</v>
+        <v>46116.29184027778</v>
       </c>
       <c r="E16">
         <v>10398</v>
@@ -4677,7 +4677,7 @@
         <v>46116.29220841435</v>
       </c>
       <c r="D17" s="1">
-        <v>46116.5421875</v>
+        <v>46116.2921875</v>
       </c>
       <c r="E17">
         <v>11094</v>
@@ -4820,7 +4820,7 @@
         <v>46116.292555706015</v>
       </c>
       <c r="D18" s="1">
-        <v>46116.54253472222</v>
+        <v>46116.29253472222</v>
       </c>
       <c r="E18">
         <v>11778</v>
@@ -4963,7 +4963,7 @@
         <v>46116.29290252315</v>
       </c>
       <c r="D19" s="1">
-        <v>46116.54288194444</v>
+        <v>46116.29288194444</v>
       </c>
       <c r="E19">
         <v>12494</v>
@@ -5106,7 +5106,7 @@
         <v>46116.293283136576</v>
       </c>
       <c r="D20" s="1">
-        <v>46116.543217592596</v>
+        <v>46116.293217592596</v>
       </c>
       <c r="E20">
         <v>13125</v>
@@ -5249,7 +5249,7 @@
         <v>46116.293249953706</v>
       </c>
       <c r="D21" s="1">
-        <v>46116.543229166666</v>
+        <v>46116.293229166666</v>
       </c>
       <c r="E21">
         <v>13218</v>
@@ -5392,7 +5392,7 @@
         <v>46116.2935975</v>
       </c>
       <c r="D22" s="1">
-        <v>46116.54357638889</v>
+        <v>46116.29357638889</v>
       </c>
       <c r="E22">
         <v>13914</v>
@@ -5535,7 +5535,7 @@
         <v>46116.2939781713</v>
       </c>
       <c r="D23" s="1">
-        <v>46116.543912037036</v>
+        <v>46116.293912037036</v>
       </c>
       <c r="E23">
         <v>14469</v>
@@ -5678,7 +5678,7 @@
         <v>46116.29394434028</v>
       </c>
       <c r="D24" s="1">
-        <v>46116.54392361111</v>
+        <v>46116.29392361111</v>
       </c>
       <c r="E24">
         <v>14582</v>
@@ -5821,7 +5821,7 @@
         <v>46116.294292280094</v>
       </c>
       <c r="D25" s="1">
-        <v>46116.544270833336</v>
+        <v>46116.294270833336</v>
       </c>
       <c r="E25">
         <v>15232</v>
@@ -5964,7 +5964,7 @@
         <v>46116.29467287037</v>
       </c>
       <c r="D26" s="1">
-        <v>46116.54460648148</v>
+        <v>46116.29460648148</v>
       </c>
       <c r="E26">
         <v>15826</v>
@@ -6107,7 +6107,7 @@
         <v>46116.29463938657</v>
       </c>
       <c r="D27" s="1">
-        <v>46116.54461805556</v>
+        <v>46116.29461805556</v>
       </c>
       <c r="E27">
         <v>15919</v>
@@ -6250,7 +6250,7 @@
         <v>46116.29498627315</v>
       </c>
       <c r="D28" s="1">
-        <v>46116.544965277775</v>
+        <v>46116.294965277775</v>
       </c>
       <c r="E28">
         <v>16626</v>
@@ -6393,7 +6393,7 @@
         <v>46116.2953671875</v>
       </c>
       <c r="D29" s="1">
-        <v>46116.54530092593</v>
+        <v>46116.29530092593</v>
       </c>
       <c r="E29">
         <v>17228</v>
@@ -6536,7 +6536,7 @@
         <v>46116.29533313657</v>
       </c>
       <c r="D30" s="1">
-        <v>46116.5453125</v>
+        <v>46116.2953125</v>
       </c>
       <c r="E30">
         <v>17322</v>
@@ -6679,7 +6679,7 @@
         <v>46116.29568109954</v>
       </c>
       <c r="D31" s="1">
-        <v>46116.54565972222</v>
+        <v>46116.29565972222</v>
       </c>
       <c r="E31">
         <v>18021</v>
@@ -6822,7 +6822,7 @@
         <v>46116.296028020835</v>
       </c>
       <c r="D32" s="1">
-        <v>46116.546006944445</v>
+        <v>46116.296006944445</v>
       </c>
       <c r="E32">
         <v>18754</v>
@@ -6965,7 +6965,7 @@
         <v>46116.29638381944</v>
       </c>
       <c r="D33" s="1">
-        <v>46116.54635416667</v>
+        <v>46116.29635416667</v>
       </c>
       <c r="E33">
         <v>19538</v>
@@ -7108,7 +7108,7 @@
         <v>46116.296747534725</v>
       </c>
       <c r="D34" s="1">
-        <v>46116.546689814815</v>
+        <v>46116.296689814815</v>
       </c>
       <c r="E34">
         <v>20188</v>
@@ -7251,7 +7251,7 @@
         <v>46116.296722210645</v>
       </c>
       <c r="D35" s="1">
-        <v>46116.54670138889</v>
+        <v>46116.29670138889</v>
       </c>
       <c r="E35">
         <v>20313</v>
@@ -7394,7 +7394,7 @@
         <v>46116.2970700463</v>
       </c>
       <c r="D36" s="1">
-        <v>46116.54704861111</v>
+        <v>46116.29704861111</v>
       </c>
       <c r="E36">
         <v>21076</v>
@@ -7537,7 +7537,7 @@
         <v>46116.2974165625</v>
       </c>
       <c r="D37" s="1">
-        <v>46116.54739583333</v>
+        <v>46116.29739583333</v>
       </c>
       <c r="E37">
         <v>21884</v>
@@ -7680,7 +7680,7 @@
         <v>46116.2977640625</v>
       </c>
       <c r="D38" s="1">
-        <v>46116.547743055555</v>
+        <v>46116.297743055555</v>
       </c>
       <c r="E38">
         <v>22679</v>
@@ -7823,7 +7823,7 @@
         <v>46116.298110972224</v>
       </c>
       <c r="D39" s="1">
-        <v>46116.54809027778</v>
+        <v>46116.29809027778</v>
       </c>
       <c r="E39">
         <v>23454</v>
@@ -7966,7 +7966,7 @@
         <v>46116.29845864583</v>
       </c>
       <c r="D40" s="1">
-        <v>46116.5484375</v>
+        <v>46116.2984375</v>
       </c>
       <c r="E40">
         <v>24189</v>
@@ -8109,7 +8109,7 @@
         <v>46116.29883939815</v>
       </c>
       <c r="D41" s="1">
-        <v>46116.54877314815</v>
+        <v>46116.29877314815</v>
       </c>
       <c r="E41">
         <v>24831</v>
@@ -8252,7 +8252,7 @@
         <v>46116.298805844905</v>
       </c>
       <c r="D42" s="1">
-        <v>46116.548784722225</v>
+        <v>46116.298784722225</v>
       </c>
       <c r="E42">
         <v>24950</v>
@@ -8395,7 +8395,7 @@
         <v>46116.29915274306</v>
       </c>
       <c r="D43" s="1">
-        <v>46116.54913194444</v>
+        <v>46116.29913194444</v>
       </c>
       <c r="E43">
         <v>25724</v>
@@ -8538,7 +8538,7 @@
         <v>46116.29953384259</v>
       </c>
       <c r="D44" s="1">
-        <v>46116.549467592595</v>
+        <v>46116.299467592595</v>
       </c>
       <c r="E44">
         <v>26372</v>
@@ -8681,7 +8681,7 @@
         <v>46116.29949996528</v>
       </c>
       <c r="D45" s="1">
-        <v>46116.549479166664</v>
+        <v>46116.299479166664</v>
       </c>
       <c r="E45">
         <v>26469</v>
@@ -8824,7 +8824,7 @@
         <v>46116.29984712963</v>
       </c>
       <c r="D46" s="1">
-        <v>46116.54982638889</v>
+        <v>46116.29982638889</v>
       </c>
       <c r="E46">
         <v>27231</v>
@@ -8967,7 +8967,7 @@
         <v>46116.30019401621</v>
       </c>
       <c r="D47" s="1">
-        <v>46116.55017361111</v>
+        <v>46116.30017361111</v>
       </c>
       <c r="E47">
         <v>28013</v>
@@ -9110,7 +9110,7 @@
         <v>46116.300542060184</v>
       </c>
       <c r="D48" s="1">
-        <v>46116.550520833334</v>
+        <v>46116.300520833334</v>
       </c>
       <c r="E48">
         <v>28808</v>
@@ -9253,7 +9253,7 @@
         <v>46116.30088891204</v>
       </c>
       <c r="D49" s="1">
-        <v>46116.55086805556</v>
+        <v>46116.30086805556</v>
       </c>
       <c r="E49">
         <v>29645</v>
@@ -9396,7 +9396,7 @@
         <v>46116.30123615741</v>
       </c>
       <c r="D50" s="1">
-        <v>46116.55121527778</v>
+        <v>46116.30121527778</v>
       </c>
       <c r="E50">
         <v>30509</v>
@@ -9539,7 +9539,7 @@
         <v>46116.30158305555</v>
       </c>
       <c r="D51" s="1">
-        <v>46116.5515625</v>
+        <v>46116.3015625</v>
       </c>
       <c r="E51">
         <v>31369</v>
@@ -9682,7 +9682,7 @@
         <v>46116.30193045139</v>
       </c>
       <c r="D52" s="1">
-        <v>46116.55190972222</v>
+        <v>46116.30190972222</v>
       </c>
       <c r="E52">
         <v>32222</v>
@@ -9825,7 +9825,7 @@
         <v>46116.3022778588</v>
       </c>
       <c r="D53" s="1">
-        <v>46116.552256944444</v>
+        <v>46116.302256944444</v>
       </c>
       <c r="E53">
         <v>33029</v>
@@ -9968,7 +9968,7 @@
         <v>46116.30262495371</v>
       </c>
       <c r="D54" s="1">
-        <v>46116.55260416667</v>
+        <v>46116.30260416667</v>
       </c>
       <c r="E54">
         <v>33689</v>
@@ -10111,7 +10111,7 @@
         <v>46116.30297179398</v>
       </c>
       <c r="D55" s="1">
-        <v>46116.55295138889</v>
+        <v>46116.30295138889</v>
       </c>
       <c r="E55">
         <v>34441</v>
@@ -10254,7 +10254,7 @@
         <v>46116.30331978009</v>
       </c>
       <c r="D56" s="1">
-        <v>46116.553298611114</v>
+        <v>46116.303298611114</v>
       </c>
       <c r="E56">
         <v>35137</v>
@@ -10397,7 +10397,7 @@
         <v>46116.30366680556</v>
       </c>
       <c r="D57" s="1">
-        <v>46116.55364583333</v>
+        <v>46116.30364583333</v>
       </c>
       <c r="E57">
         <v>35892</v>
@@ -10540,7 +10540,7 @@
         <v>46116.30401359954</v>
       </c>
       <c r="D58" s="1">
-        <v>46116.55399305555</v>
+        <v>46116.30399305555</v>
       </c>
       <c r="E58">
         <v>36696</v>
@@ -10683,7 +10683,7 @@
         <v>46116.30436045139</v>
       </c>
       <c r="D59" s="1">
-        <v>46116.55434027778</v>
+        <v>46116.30434027778</v>
       </c>
       <c r="E59">
         <v>37597</v>
@@ -10826,7 +10826,7 @@
         <v>46116.304708171294</v>
       </c>
       <c r="D60" s="1">
-        <v>46116.5546875</v>
+        <v>46116.3046875</v>
       </c>
       <c r="E60">
         <v>38548</v>
@@ -10969,7 +10969,7 @@
         <v>46116.30505545139</v>
       </c>
       <c r="D61" s="1">
-        <v>46116.55503472222</v>
+        <v>46116.30503472222</v>
       </c>
       <c r="E61">
         <v>39576</v>
@@ -11112,7 +11112,7 @@
         <v>46116.30540292824</v>
       </c>
       <c r="D62" s="1">
-        <v>46116.55538194445</v>
+        <v>46116.30538194445</v>
       </c>
       <c r="E62">
         <v>40554</v>
@@ -11255,7 +11255,7 @@
         <v>46116.30574957176</v>
       </c>
       <c r="D63" s="1">
-        <v>46116.55572916667</v>
+        <v>46116.30572916667</v>
       </c>
       <c r="E63">
         <v>41508</v>
@@ -11398,7 +11398,7 @@
         <v>46116.30609709491</v>
       </c>
       <c r="D64" s="1">
-        <v>46116.556076388886</v>
+        <v>46116.306076388886</v>
       </c>
       <c r="E64">
         <v>42311</v>
@@ -11541,7 +11541,7 @@
         <v>46116.30645241898</v>
       </c>
       <c r="D65" s="1">
-        <v>46116.55642361111</v>
+        <v>46116.30642361111</v>
       </c>
       <c r="E65">
         <v>42856</v>
@@ -11684,7 +11684,7 @@
         <v>46116.30678861111</v>
       </c>
       <c r="D66" s="1">
-        <v>46116.556759259256</v>
+        <v>46116.306759259256</v>
       </c>
       <c r="E66">
         <v>43096</v>
@@ -11827,7 +11827,7 @@
         <v>46116.306791469906</v>
       </c>
       <c r="D67" s="1">
-        <v>46116.55677083333</v>
+        <v>46116.30677083333</v>
       </c>
       <c r="E67">
         <v>43177</v>
@@ -11970,7 +11970,7 @@
         <v>46116.30716502315</v>
       </c>
       <c r="D68" s="1">
-        <v>46116.55710648148</v>
+        <v>46116.30710648148</v>
       </c>
       <c r="E68">
         <v>43692</v>
@@ -12113,7 +12113,7 @@
         <v>46116.30713861111</v>
       </c>
       <c r="D69" s="1">
-        <v>46116.557118055556</v>
+        <v>46116.307118055556</v>
       </c>
       <c r="E69">
         <v>43787</v>
@@ -12256,7 +12256,7 @@
         <v>46116.30748596065</v>
       </c>
       <c r="D70" s="1">
-        <v>46116.55746527778</v>
+        <v>46116.30746527778</v>
       </c>
       <c r="E70">
         <v>44438</v>
@@ -12399,7 +12399,7 @@
         <v>46116.30785903935</v>
       </c>
       <c r="D71" s="1">
-        <v>46116.557800925926</v>
+        <v>46116.307800925926</v>
       </c>
       <c r="E71">
         <v>45094</v>
@@ -12542,7 +12542,7 @@
         <v>46116.30783329861</v>
       </c>
       <c r="D72" s="1">
-        <v>46116.5578125</v>
+        <v>46116.3078125</v>
       </c>
       <c r="E72">
         <v>45184</v>
@@ -12685,7 +12685,7 @@
         <v>46116.30817761574</v>
       </c>
       <c r="D73" s="1">
-        <v>46116.55814814815</v>
+        <v>46116.30814814815</v>
       </c>
       <c r="E73">
         <v>45719</v>
@@ -12828,7 +12828,7 @@
         <v>46116.308180625</v>
       </c>
       <c r="D74" s="1">
-        <v>46116.55815972222</v>
+        <v>46116.30815972222</v>
       </c>
       <c r="E74">
         <v>45814</v>
@@ -12971,7 +12971,7 @@
         <v>46116.308527824076</v>
       </c>
       <c r="D75" s="1">
-        <v>46116.55850694444</v>
+        <v>46116.30850694444</v>
       </c>
       <c r="E75">
         <v>46695</v>
@@ -13114,7 +13114,7 @@
         <v>46116.30887435185</v>
       </c>
       <c r="D76" s="1">
-        <v>46116.558854166666</v>
+        <v>46116.308854166666</v>
       </c>
       <c r="E76">
         <v>47610</v>
@@ -13257,7 +13257,7 @@
         <v>46116.309221689815</v>
       </c>
       <c r="D77" s="1">
-        <v>46116.55920138889</v>
+        <v>46116.30920138889</v>
       </c>
       <c r="E77">
         <v>48563</v>
@@ -13400,7 +13400,7 @@
         <v>46116.30956944444</v>
       </c>
       <c r="D78" s="1">
-        <v>46116.55954861111</v>
+        <v>46116.30954861111</v>
       </c>
       <c r="E78">
         <v>49436</v>
@@ -13543,7 +13543,7 @@
         <v>46116.30991672454</v>
       </c>
       <c r="D79" s="1">
-        <v>46116.559895833336</v>
+        <v>46116.309895833336</v>
       </c>
       <c r="E79">
         <v>50346</v>
@@ -13686,7 +13686,7 @@
         <v>46116.31026358796</v>
       </c>
       <c r="D80" s="1">
-        <v>46116.56024305556</v>
+        <v>46116.31024305556</v>
       </c>
       <c r="E80">
         <v>51196</v>
@@ -13829,7 +13829,7 @@
         <v>46116.31061091435</v>
       </c>
       <c r="D81" s="1">
-        <v>46116.560590277775</v>
+        <v>46116.310590277775</v>
       </c>
       <c r="E81">
         <v>51974</v>
@@ -13972,7 +13972,7 @@
         <v>46116.31095818287</v>
       </c>
       <c r="D82" s="1">
-        <v>46116.5609375</v>
+        <v>46116.3109375</v>
       </c>
       <c r="E82">
         <v>52816</v>
@@ -14115,7 +14115,7 @@
         <v>46116.311305428244</v>
       </c>
       <c r="D83" s="1">
-        <v>46116.56128472222</v>
+        <v>46116.31128472222</v>
       </c>
       <c r="E83">
         <v>53302</v>
@@ -14258,7 +14258,7 @@
         <v>46116.311652523145</v>
       </c>
       <c r="D84" s="1">
-        <v>46116.561631944445</v>
+        <v>46116.311631944445</v>
       </c>
       <c r="E84">
         <v>53912</v>
@@ -14401,7 +14401,7 @@
         <v>46116.312008125</v>
       </c>
       <c r="D85" s="1">
-        <v>46116.56197916667</v>
+        <v>46116.31197916667</v>
       </c>
       <c r="E85">
         <v>54736</v>
@@ -14544,7 +14544,7 @@
         <v>46116.31234636574</v>
       </c>
       <c r="D86" s="1">
-        <v>46116.56232638889</v>
+        <v>46116.31232638889</v>
       </c>
       <c r="E86">
         <v>55628</v>
@@ -14687,7 +14687,7 @@
         <v>46116.31269359954</v>
       </c>
       <c r="D87" s="1">
-        <v>46116.56267361111</v>
+        <v>46116.31267361111</v>
       </c>
       <c r="E87">
         <v>56163</v>
@@ -14830,7 +14830,7 @@
         <v>46116.31305009259</v>
       </c>
       <c r="D88" s="1">
-        <v>46116.56302083333</v>
+        <v>46116.31302083333</v>
       </c>
       <c r="E88">
         <v>56761</v>
@@ -14973,7 +14973,7 @@
         <v>46116.31338821759</v>
       </c>
       <c r="D89" s="1">
-        <v>46116.563368055555</v>
+        <v>46116.313368055555</v>
       </c>
       <c r="E89">
         <v>57481</v>
@@ -15116,7 +15116,7 @@
         <v>46116.313736006945</v>
       </c>
       <c r="D90" s="1">
-        <v>46116.56371527778</v>
+        <v>46116.31371527778</v>
       </c>
       <c r="E90">
         <v>58392</v>
@@ -15262,7 +15262,7 @@
         <v>46116.31408333333</v>
       </c>
       <c r="D91" s="1">
-        <v>46116.5640625</v>
+        <v>46116.3140625</v>
       </c>
       <c r="E91">
         <v>58995</v>
@@ -15405,7 +15405,7 @@
         <v>46116.31443020833</v>
       </c>
       <c r="D92" s="1">
-        <v>46116.564409722225</v>
+        <v>46116.314409722225</v>
       </c>
       <c r="E92">
         <v>59727</v>
@@ -15548,7 +15548,7 @@
         <v>46116.31477755787</v>
       </c>
       <c r="D93" s="1">
-        <v>46116.56475694444</v>
+        <v>46116.31475694444</v>
       </c>
       <c r="E93">
         <v>60359</v>
@@ -15691,7 +15691,7 @@
         <v>46116.31512428241</v>
       </c>
       <c r="D94" s="1">
-        <v>46116.565104166664</v>
+        <v>46116.315104166664</v>
       </c>
       <c r="E94">
         <v>60784</v>
@@ -15834,7 +15834,7 @@
         <v>46116.31547184028</v>
       </c>
       <c r="D95" s="1">
-        <v>46116.56545138889</v>
+        <v>46116.31545138889</v>
       </c>
       <c r="E95">
         <v>61238</v>
@@ -15977,7 +15977,7 @@
         <v>46116.31581923611</v>
       </c>
       <c r="D96" s="1">
-        <v>46116.56579861111</v>
+        <v>46116.31579861111</v>
       </c>
       <c r="E96">
         <v>61705</v>
@@ -16120,7 +16120,7 @@
         <v>46116.31616618056</v>
       </c>
       <c r="D97" s="1">
-        <v>46116.566145833334</v>
+        <v>46116.316145833334</v>
       </c>
       <c r="E97">
         <v>62533</v>
@@ -16263,7 +16263,7 @@
         <v>46116.31651386574</v>
       </c>
       <c r="D98" s="1">
-        <v>46116.56649305556</v>
+        <v>46116.31649305556</v>
       </c>
       <c r="E98">
         <v>63441</v>
@@ -16406,7 +16406,7 @@
         <v>46116.31686075231</v>
       </c>
       <c r="D99" s="1">
-        <v>46116.56684027778</v>
+        <v>46116.31684027778</v>
       </c>
       <c r="E99">
         <v>64392</v>
@@ -16549,7 +16549,7 @@
         <v>46116.317208229164</v>
       </c>
       <c r="D100" s="1">
-        <v>46116.5671875</v>
+        <v>46116.3171875</v>
       </c>
       <c r="E100">
         <v>64939</v>
@@ -16692,7 +16692,7 @@
         <v>46116.31755519676</v>
       </c>
       <c r="D101" s="1">
-        <v>46116.56753472222</v>
+        <v>46116.31753472222</v>
       </c>
       <c r="E101">
         <v>65452</v>
@@ -16835,7 +16835,7 @@
         <v>46116.31790274305</v>
       </c>
       <c r="D102" s="1">
-        <v>46116.567881944444</v>
+        <v>46116.317881944444</v>
       </c>
       <c r="E102">
         <v>65940</v>
@@ -16978,7 +16978,7 @@
         <v>46116.3182496875</v>
       </c>
       <c r="D103" s="1">
-        <v>46116.56822916667</v>
+        <v>46116.31822916667</v>
       </c>
       <c r="E103">
         <v>66366</v>
@@ -17121,7 +17121,7 @@
         <v>46116.3185971412</v>
       </c>
       <c r="D104" s="1">
-        <v>46116.56857638889</v>
+        <v>46116.31857638889</v>
       </c>
       <c r="E104">
         <v>66866</v>
@@ -17264,7 +17264,7 @@
         <v>46116.31894424769</v>
       </c>
       <c r="D105" s="1">
-        <v>46116.568923611114</v>
+        <v>46116.318923611114</v>
       </c>
       <c r="E105">
         <v>67366</v>
@@ -17407,7 +17407,7 @@
         <v>46116.31929172454</v>
       </c>
       <c r="D106" s="1">
-        <v>46116.56927083333</v>
+        <v>46116.31927083333</v>
       </c>
       <c r="E106">
         <v>67887</v>
@@ -17550,7 +17550,7 @@
         <v>46116.319638877314</v>
       </c>
       <c r="D107" s="1">
-        <v>46116.56961805555</v>
+        <v>46116.31961805555</v>
       </c>
       <c r="E107">
         <v>68401</v>
@@ -17693,7 +17693,7 @@
         <v>46116.319985821756</v>
       </c>
       <c r="D108" s="1">
-        <v>46116.56996527778</v>
+        <v>46116.31996527778</v>
       </c>
       <c r="E108">
         <v>68874</v>
@@ -17836,7 +17836,7 @@
         <v>46116.32033314815</v>
       </c>
       <c r="D109" s="1">
-        <v>46116.5703125</v>
+        <v>46116.3203125</v>
       </c>
       <c r="E109">
         <v>69368</v>
@@ -17979,7 +17979,7 @@
         <v>46116.320680439814</v>
       </c>
       <c r="D110" s="1">
-        <v>46116.57065972222</v>
+        <v>46116.32065972222</v>
       </c>
       <c r="E110">
         <v>69819</v>
@@ -18122,7 +18122,7 @@
         <v>46116.321027199076</v>
       </c>
       <c r="D111" s="1">
-        <v>46116.57100694445</v>
+        <v>46116.32100694445</v>
       </c>
       <c r="E111">
         <v>70416</v>
@@ -18265,7 +18265,7 @@
         <v>46116.321374976855</v>
       </c>
       <c r="D112" s="1">
-        <v>46116.57135416667</v>
+        <v>46116.32135416667</v>
       </c>
       <c r="E112">
         <v>70957</v>
@@ -18408,7 +18408,7 @@
         <v>46116.32172247685</v>
       </c>
       <c r="D113" s="1">
-        <v>46116.571701388886</v>
+        <v>46116.321701388886</v>
       </c>
       <c r="E113">
         <v>71383</v>
@@ -18551,7 +18551,7 @@
         <v>46116.32207785879</v>
       </c>
       <c r="D114" s="1">
-        <v>46116.57204861111</v>
+        <v>46116.32204861111</v>
       </c>
       <c r="E114">
         <v>72076</v>
@@ -18694,7 +18694,7 @@
         <v>46116.322425011575</v>
       </c>
       <c r="D115" s="1">
-        <v>46116.57239583333</v>
+        <v>46116.32239583333</v>
       </c>
       <c r="E115">
         <v>72587</v>
@@ -18837,7 +18837,7 @@
         <v>46116.32276434028</v>
       </c>
       <c r="D116" s="1">
-        <v>46116.572743055556</v>
+        <v>46116.322743055556</v>
       </c>
       <c r="E116">
         <v>73156</v>
@@ -18980,7 +18980,7 @@
         <v>46116.323109606485</v>
       </c>
       <c r="D117" s="1">
-        <v>46116.57309027778</v>
+        <v>46116.32309027778</v>
       </c>
       <c r="E117">
         <v>73735</v>
@@ -19123,7 +19123,7 @@
         <v>46116.32345858796</v>
       </c>
       <c r="D118" s="1">
-        <v>46116.5734375</v>
+        <v>46116.3234375</v>
       </c>
       <c r="E118">
         <v>74362</v>
@@ -19266,7 +19266,7 @@
         <v>46116.32380537037</v>
       </c>
       <c r="D119" s="1">
-        <v>46116.57378472222</v>
+        <v>46116.32378472222</v>
       </c>
       <c r="E119">
         <v>74890</v>
@@ -19409,7 +19409,7 @@
         <v>46116.32415287037</v>
       </c>
       <c r="D120" s="1">
-        <v>46116.57413194444</v>
+        <v>46116.32413194444</v>
       </c>
       <c r="E120">
         <v>75384</v>
@@ -19552,7 +19552,7 @@
         <v>46116.32449998843</v>
       </c>
       <c r="D121" s="1">
-        <v>46116.574479166666</v>
+        <v>46116.324479166666</v>
       </c>
       <c r="E121">
         <v>75894</v>
@@ -19695,7 +19695,7 @@
         <v>46116.32484758102</v>
       </c>
       <c r="D122" s="1">
-        <v>46116.57482638889</v>
+        <v>46116.32482638889</v>
       </c>
       <c r="E122">
         <v>76378</v>
@@ -19838,7 +19838,7 @@
         <v>46116.32519434028</v>
       </c>
       <c r="D123" s="1">
-        <v>46116.57517361111</v>
+        <v>46116.32517361111</v>
       </c>
       <c r="E123">
         <v>76951</v>
@@ -19981,7 +19981,7 @@
         <v>46116.32554158565</v>
       </c>
       <c r="D124" s="1">
-        <v>46116.575520833336</v>
+        <v>46116.325520833336</v>
       </c>
       <c r="E124">
         <v>77575</v>
@@ -20124,7 +20124,7 @@
         <v>46116.325914560184</v>
       </c>
       <c r="D125" s="1">
-        <v>46116.57585648148</v>
+        <v>46116.32585648148</v>
       </c>
       <c r="E125">
         <v>78056</v>
@@ -20267,7 +20267,7 @@
         <v>46116.32588885417</v>
       </c>
       <c r="D126" s="1">
-        <v>46116.57586805556</v>
+        <v>46116.32586805556</v>
       </c>
       <c r="E126">
         <v>78136</v>
@@ -20410,7 +20410,7 @@
         <v>46116.32623564815</v>
       </c>
       <c r="D127" s="1">
-        <v>46116.576215277775</v>
+        <v>46116.326215277775</v>
       </c>
       <c r="E127">
         <v>78644</v>
@@ -20553,7 +20553,7 @@
         <v>46116.32658310185</v>
       </c>
       <c r="D128" s="1">
-        <v>46116.5765625</v>
+        <v>46116.3265625</v>
       </c>
       <c r="E128">
         <v>79171</v>
@@ -20696,7 +20696,7 @@
         <v>46116.32692986111</v>
       </c>
       <c r="D129" s="1">
-        <v>46116.57690972222</v>
+        <v>46116.32690972222</v>
       </c>
       <c r="E129">
         <v>79678</v>
@@ -20839,7 +20839,7 @@
         <v>46116.32727800926</v>
       </c>
       <c r="D130" s="1">
-        <v>46116.577256944445</v>
+        <v>46116.327256944445</v>
       </c>
       <c r="E130">
         <v>80199</v>
@@ -20982,7 +20982,7 @@
         <v>46116.327624398145</v>
       </c>
       <c r="D131" s="1">
-        <v>46116.57760416667</v>
+        <v>46116.32760416667</v>
       </c>
       <c r="E131">
         <v>80706</v>
@@ -21125,7 +21125,7 @@
         <v>46116.3280066088</v>
       </c>
       <c r="D132" s="1">
-        <v>46116.577939814815</v>
+        <v>46116.327939814815</v>
       </c>
       <c r="E132">
         <v>81116</v>
@@ -21268,7 +21268,7 @@
         <v>46116.327972175925</v>
       </c>
       <c r="D133" s="1">
-        <v>46116.57795138889</v>
+        <v>46116.32795138889</v>
       </c>
       <c r="E133">
         <v>81196</v>
@@ -21411,7 +21411,7 @@
         <v>46116.32831943287</v>
       </c>
       <c r="D134" s="1">
-        <v>46116.57829861111</v>
+        <v>46116.32829861111</v>
       </c>
       <c r="E134">
         <v>81714</v>
@@ -21554,7 +21554,7 @@
         <v>46116.32866638889</v>
       </c>
       <c r="D135" s="1">
-        <v>46116.57864583333</v>
+        <v>46116.32864583333</v>
       </c>
       <c r="E135">
         <v>82205</v>
@@ -21697,7 +21697,7 @@
         <v>46116.329013518516</v>
       </c>
       <c r="D136" s="1">
-        <v>46116.578993055555</v>
+        <v>46116.328993055555</v>
       </c>
       <c r="E136">
         <v>82699</v>
@@ -21840,7 +21840,7 @@
         <v>46116.32936119213</v>
       </c>
       <c r="D137" s="1">
-        <v>46116.57934027778</v>
+        <v>46116.32934027778</v>
       </c>
       <c r="E137">
         <v>83196</v>
@@ -21983,7 +21983,7 @@
         <v>46116.3297137037</v>
       </c>
       <c r="D138" s="1">
-        <v>46116.579675925925</v>
+        <v>46116.329675925925</v>
       </c>
       <c r="E138">
         <v>83631</v>
@@ -22126,7 +22126,7 @@
         <v>46116.32971126158</v>
       </c>
       <c r="D139" s="1">
-        <v>46116.5796875</v>
+        <v>46116.3296875</v>
       </c>
       <c r="E139">
         <v>83715</v>
@@ -22269,7 +22269,7 @@
         <v>46116.330090219904</v>
       </c>
       <c r="D140" s="1">
-        <v>46116.58002314815</v>
+        <v>46116.33002314815</v>
       </c>
       <c r="E140">
         <v>84198</v>
@@ -22412,7 +22412,7 @@
         <v>46116.330055162034</v>
       </c>
       <c r="D141" s="1">
-        <v>46116.580034722225</v>
+        <v>46116.330034722225</v>
       </c>
       <c r="E141">
         <v>84283</v>
@@ -22711,7 +22711,7 @@
         <v>46116.33040542824</v>
       </c>
       <c r="D2" s="1">
-        <v>46116.58038194444</v>
+        <v>46116.33038194444</v>
       </c>
       <c r="E2">
         <v>82796</v>
@@ -22818,7 +22818,7 @@
         <v>46116.33075047454</v>
       </c>
       <c r="D3" s="1">
-        <v>46116.580729166664</v>
+        <v>46116.330729166664</v>
       </c>
       <c r="E3">
         <v>79737</v>
@@ -22949,7 +22949,7 @@
         <v>46116.33109675926</v>
       </c>
       <c r="D4" s="1">
-        <v>46116.58107638889</v>
+        <v>46116.33107638889</v>
       </c>
       <c r="E4">
         <v>76939</v>
@@ -23092,7 +23092,7 @@
         <v>46116.33144440972</v>
       </c>
       <c r="D5" s="1">
-        <v>46116.58142361111</v>
+        <v>46116.33142361111</v>
       </c>
       <c r="E5">
         <v>74298</v>
@@ -23235,7 +23235,7 @@
         <v>46116.33179457176</v>
       </c>
       <c r="D6" s="1">
-        <v>46116.581770833334</v>
+        <v>46116.331770833334</v>
       </c>
       <c r="E6">
         <v>71778</v>
@@ -23378,7 +23378,7 @@
         <v>46116.33213888889</v>
       </c>
       <c r="D7" s="1">
-        <v>46116.58211805556</v>
+        <v>46116.33211805556</v>
       </c>
       <c r="E7">
         <v>69423</v>
@@ -23521,7 +23521,7 @@
         <v>46116.33248560185</v>
       </c>
       <c r="D8" s="1">
-        <v>46116.58246527778</v>
+        <v>46116.33246527778</v>
       </c>
       <c r="E8">
         <v>67182</v>
@@ -23664,7 +23664,7 @@
         <v>46116.33283313658</v>
       </c>
       <c r="D9" s="1">
-        <v>46116.5828125</v>
+        <v>46116.3328125</v>
       </c>
       <c r="E9">
         <v>65044</v>
@@ -23807,7 +23807,7 @@
         <v>46116.33318304398</v>
       </c>
       <c r="D10" s="1">
-        <v>46116.58315972222</v>
+        <v>46116.33315972222</v>
       </c>
       <c r="E10">
         <v>63121</v>
@@ -23950,7 +23950,7 @@
         <v>46116.333527766204</v>
       </c>
       <c r="D11" s="1">
-        <v>46116.583506944444</v>
+        <v>46116.333506944444</v>
       </c>
       <c r="E11">
         <v>61325</v>
@@ -24093,7 +24093,7 @@
         <v>46116.333877523146</v>
       </c>
       <c r="D12" s="1">
-        <v>46116.58385416667</v>
+        <v>46116.33385416667</v>
       </c>
       <c r="E12">
         <v>59785</v>
@@ -24236,7 +24236,7 @@
         <v>46116.334222164354</v>
       </c>
       <c r="D13" s="1">
-        <v>46116.58420138889</v>
+        <v>46116.33420138889</v>
       </c>
       <c r="E13">
         <v>58269</v>
@@ -24379,7 +24379,7 @@
         <v>46116.33457886574</v>
       </c>
       <c r="D14" s="1">
-        <v>46116.584548611114</v>
+        <v>46116.334548611114</v>
       </c>
       <c r="E14">
         <v>56716</v>
@@ -24522,7 +24522,7 @@
         <v>46116.33491643518</v>
       </c>
       <c r="D15" s="1">
-        <v>46116.58489583333</v>
+        <v>46116.33489583333</v>
       </c>
       <c r="E15">
         <v>55059</v>
@@ -24665,7 +24665,7 @@
         <v>46116.33526361111</v>
       </c>
       <c r="D16" s="1">
-        <v>46116.58524305555</v>
+        <v>46116.33524305555</v>
       </c>
       <c r="E16">
         <v>53569</v>
@@ -24808,7 +24808,7 @@
         <v>46116.33561144676</v>
       </c>
       <c r="D17" s="1">
-        <v>46116.58559027778</v>
+        <v>46116.33559027778</v>
       </c>
       <c r="E17">
         <v>52346</v>
@@ -24951,7 +24951,7 @@
         <v>46116.335960254626</v>
       </c>
       <c r="D18" s="1">
-        <v>46116.5859375</v>
+        <v>46116.3359375</v>
       </c>
       <c r="E18">
         <v>51166</v>
@@ -25094,7 +25094,7 @@
         <v>46116.33630836805</v>
       </c>
       <c r="D19" s="1">
-        <v>46116.58628472222</v>
+        <v>46116.33628472222</v>
       </c>
       <c r="E19">
         <v>49933</v>
@@ -25237,7 +25237,7 @@
         <v>46116.33665280093</v>
       </c>
       <c r="D20" s="1">
-        <v>46116.58663194445</v>
+        <v>46116.33663194445</v>
       </c>
       <c r="E20">
         <v>48745</v>
@@ -25380,7 +25380,7 @@
         <v>46116.33699952546</v>
       </c>
       <c r="D21" s="1">
-        <v>46116.58697916667</v>
+        <v>46116.33697916667</v>
       </c>
       <c r="E21">
         <v>47637</v>
@@ -25523,7 +25523,7 @@
         <v>46116.33735094908</v>
       </c>
       <c r="D22" s="1">
-        <v>46116.587326388886</v>
+        <v>46116.337326388886</v>
       </c>
       <c r="E22">
         <v>46555</v>
@@ -25666,7 +25666,7 @@
         <v>46116.33769606482</v>
       </c>
       <c r="D23" s="1">
-        <v>46116.58767361111</v>
+        <v>46116.33767361111</v>
       </c>
       <c r="E23">
         <v>45464</v>
@@ -25809,7 +25809,7 @@
         <v>46116.338042048614</v>
       </c>
       <c r="D24" s="1">
-        <v>46116.58802083333</v>
+        <v>46116.33802083333</v>
       </c>
       <c r="E24">
         <v>44364</v>
@@ -25952,7 +25952,7 @@
         <v>46116.338389386576</v>
       </c>
       <c r="D25" s="1">
-        <v>46116.588368055556</v>
+        <v>46116.338368055556</v>
       </c>
       <c r="E25">
         <v>43316</v>
@@ -26095,7 +26095,7 @@
         <v>46116.33873633102</v>
       </c>
       <c r="D26" s="1">
-        <v>46116.58871527778</v>
+        <v>46116.33871527778</v>
       </c>
       <c r="E26">
         <v>42272</v>
@@ -26238,7 +26238,7 @@
         <v>46116.339083101855</v>
       </c>
       <c r="D27" s="1">
-        <v>46116.5890625</v>
+        <v>46116.3390625</v>
       </c>
       <c r="E27">
         <v>41268</v>
@@ -26381,7 +26381,7 @@
         <v>46116.339433402776</v>
       </c>
       <c r="D28" s="1">
-        <v>46116.58940972222</v>
+        <v>46116.33940972222</v>
       </c>
       <c r="E28">
         <v>40330</v>
@@ -26524,7 +26524,7 @@
         <v>46116.33978116898</v>
       </c>
       <c r="D29" s="1">
-        <v>46116.58975694444</v>
+        <v>46116.33975694444</v>
       </c>
       <c r="E29">
         <v>39454</v>
@@ -26667,7 +26667,7 @@
         <v>46116.3401278588</v>
       </c>
       <c r="D30" s="1">
-        <v>46116.590104166666</v>
+        <v>46116.340104166666</v>
       </c>
       <c r="E30">
         <v>38549</v>
@@ -26810,7 +26810,7 @@
         <v>46116.34047258102</v>
       </c>
       <c r="D31" s="1">
-        <v>46116.59045138889</v>
+        <v>46116.34045138889</v>
       </c>
       <c r="E31">
         <v>37611</v>
@@ -26953,7 +26953,7 @@
         <v>46116.34081931713</v>
       </c>
       <c r="D32" s="1">
-        <v>46116.59079861111</v>
+        <v>46116.34079861111</v>
       </c>
       <c r="E32">
         <v>36652</v>
@@ -27096,7 +27096,7 @@
         <v>46116.341166018516</v>
       </c>
       <c r="D33" s="1">
-        <v>46116.591145833336</v>
+        <v>46116.341145833336</v>
       </c>
       <c r="E33">
         <v>35701</v>
@@ -27239,7 +27239,7 @@
         <v>46116.34151388889</v>
       </c>
       <c r="D34" s="1">
-        <v>46116.59149305556</v>
+        <v>46116.34149305556</v>
       </c>
       <c r="E34">
         <v>34822</v>
@@ -27382,7 +27382,7 @@
         <v>46116.34186184028</v>
       </c>
       <c r="D35" s="1">
-        <v>46116.591840277775</v>
+        <v>46116.341840277775</v>
       </c>
       <c r="E35">
         <v>33955</v>
@@ -27525,7 +27525,7 @@
         <v>46116.3422112037</v>
       </c>
       <c r="D36" s="1">
-        <v>46116.5921875</v>
+        <v>46116.3421875</v>
       </c>
       <c r="E36">
         <v>33119</v>
@@ -27668,7 +27668,7 @@
         <v>46116.34258885417</v>
       </c>
       <c r="D37" s="1">
-        <v>46116.592523148145</v>
+        <v>46116.342523148145</v>
       </c>
       <c r="E37">
         <v>32290</v>
@@ -27811,7 +27811,7 @@
         <v>46116.34255934028</v>
       </c>
       <c r="D38" s="1">
-        <v>46116.59253472222</v>
+        <v>46116.34253472222</v>
       </c>
       <c r="E38">
         <v>32283</v>
@@ -27954,7 +27954,7 @@
         <v>46116.342904756944</v>
       </c>
       <c r="D39" s="1">
-        <v>46116.592881944445</v>
+        <v>46116.342881944445</v>
       </c>
       <c r="E39">
         <v>31437</v>
@@ -28097,7 +28097,7 @@
         <v>46116.34325099537</v>
       </c>
       <c r="D40" s="1">
-        <v>46116.59322916667</v>
+        <v>46116.34322916667</v>
       </c>
       <c r="E40">
         <v>30643</v>
@@ -28240,7 +28240,7 @@
         <v>46116.34360371528</v>
       </c>
       <c r="D41" s="1">
-        <v>46116.593564814815</v>
+        <v>46116.343564814815</v>
       </c>
       <c r="E41">
         <v>29815</v>
@@ -28383,7 +28383,7 @@
         <v>46116.343599768516</v>
       </c>
       <c r="D42" s="1">
-        <v>46116.59357638889</v>
+        <v>46116.34357638889</v>
       </c>
       <c r="E42">
         <v>29854</v>
@@ -28526,7 +28526,7 @@
         <v>46116.34397918981</v>
       </c>
       <c r="D43" s="1">
-        <v>46116.59391203704</v>
+        <v>46116.34391203704</v>
       </c>
       <c r="E43">
         <v>29055</v>
@@ -28669,7 +28669,7 @@
         <v>46116.34394438657</v>
       </c>
       <c r="D44" s="1">
-        <v>46116.59392361111</v>
+        <v>46116.34392361111</v>
       </c>
       <c r="E44">
         <v>29098</v>
@@ -28812,7 +28812,7 @@
         <v>46116.34429224537</v>
       </c>
       <c r="D45" s="1">
-        <v>46116.59427083333</v>
+        <v>46116.34427083333</v>
       </c>
       <c r="E45">
         <v>28329</v>
@@ -28955,7 +28955,7 @@
         <v>46116.34463863426</v>
       </c>
       <c r="D46" s="1">
-        <v>46116.594618055555</v>
+        <v>46116.344618055555</v>
       </c>
       <c r="E46">
         <v>27561</v>
@@ -29098,7 +29098,7 @@
         <v>46116.3449890162</v>
       </c>
       <c r="D47" s="1">
-        <v>46116.59496527778</v>
+        <v>46116.34496527778</v>
       </c>
       <c r="E47">
         <v>26829</v>
@@ -29241,7 +29241,7 @@
         <v>46116.3453330787</v>
       </c>
       <c r="D48" s="1">
-        <v>46116.5953125</v>
+        <v>46116.3453125</v>
       </c>
       <c r="E48">
         <v>26083</v>
@@ -29384,7 +29384,7 @@
         <v>46116.34568248843</v>
       </c>
       <c r="D49" s="1">
-        <v>46116.595659722225</v>
+        <v>46116.345659722225</v>
       </c>
       <c r="E49">
         <v>25313</v>
@@ -29527,7 +29527,7 @@
         <v>46116.34602822916</v>
       </c>
       <c r="D50" s="1">
-        <v>46116.59600694444</v>
+        <v>46116.34600694444</v>
       </c>
       <c r="E50">
         <v>24587</v>
@@ -29670,7 +29670,7 @@
         <v>46116.34637489583</v>
       </c>
       <c r="D51" s="1">
-        <v>46116.596354166664</v>
+        <v>46116.346354166664</v>
       </c>
       <c r="E51">
         <v>23868</v>
@@ -29813,7 +29813,7 @@
         <v>46116.34672167824</v>
       </c>
       <c r="D52" s="1">
-        <v>46116.59670138889</v>
+        <v>46116.34670138889</v>
       </c>
       <c r="E52">
         <v>23139</v>
@@ -29956,7 +29956,7 @@
         <v>46116.34706949074</v>
       </c>
       <c r="D53" s="1">
-        <v>46116.59704861111</v>
+        <v>46116.34704861111</v>
       </c>
       <c r="E53">
         <v>22457</v>
@@ -30099,7 +30099,7 @@
         <v>46116.34745180556</v>
       </c>
       <c r="D54" s="1">
-        <v>46116.59738425926</v>
+        <v>46116.34738425926</v>
       </c>
       <c r="E54">
         <v>21732</v>
@@ -30242,7 +30242,7 @@
         <v>46116.34741633102</v>
       </c>
       <c r="D55" s="1">
-        <v>46116.597395833334</v>
+        <v>46116.347395833334</v>
       </c>
       <c r="E55">
         <v>21771</v>
@@ -30385,7 +30385,7 @@
         <v>46116.347766631945</v>
       </c>
       <c r="D56" s="1">
-        <v>46116.59774305556</v>
+        <v>46116.34774305556</v>
       </c>
       <c r="E56">
         <v>21093</v>
@@ -30528,7 +30528,7 @@
         <v>46116.34814765046</v>
       </c>
       <c r="D57" s="1">
-        <v>46116.598078703704</v>
+        <v>46116.348078703704</v>
       </c>
       <c r="E57">
         <v>20412</v>
@@ -30671,7 +30671,7 @@
         <v>46116.348111342595</v>
       </c>
       <c r="D58" s="1">
-        <v>46116.59809027778</v>
+        <v>46116.34809027778</v>
       </c>
       <c r="E58">
         <v>20431</v>
@@ -30814,7 +30814,7 @@
         <v>46116.34845923611</v>
       </c>
       <c r="D59" s="1">
-        <v>46116.5984375</v>
+        <v>46116.3484375</v>
       </c>
       <c r="E59">
         <v>19780</v>
@@ -30957,7 +30957,7 @@
         <v>46116.348836157405</v>
       </c>
       <c r="D60" s="1">
-        <v>46116.59877314815</v>
+        <v>46116.34877314815</v>
       </c>
       <c r="E60">
         <v>19101</v>
@@ -31100,7 +31100,7 @@
         <v>46116.34880594908</v>
       </c>
       <c r="D61" s="1">
-        <v>46116.59878472222</v>
+        <v>46116.34878472222</v>
       </c>
       <c r="E61">
         <v>19145</v>
@@ -31243,7 +31243,7 @@
         <v>46116.349155208336</v>
       </c>
       <c r="D62" s="1">
-        <v>46116.599131944444</v>
+        <v>46116.349131944444</v>
       </c>
       <c r="E62">
         <v>18533</v>
@@ -31386,7 +31386,7 @@
         <v>46116.3495303125</v>
       </c>
       <c r="D63" s="1">
-        <v>46116.59946759259</v>
+        <v>46116.34946759259</v>
       </c>
       <c r="E63">
         <v>17887</v>
@@ -31529,7 +31529,7 @@
         <v>46116.3495012037</v>
       </c>
       <c r="D64" s="1">
-        <v>46116.59947916667</v>
+        <v>46116.34947916667</v>
       </c>
       <c r="E64">
         <v>17930</v>
@@ -31672,7 +31672,7 @@
         <v>46116.34984782407</v>
       </c>
       <c r="D65" s="1">
-        <v>46116.59982638889</v>
+        <v>46116.34982638889</v>
       </c>
       <c r="E65">
         <v>17330</v>
@@ -31815,7 +31815,7 @@
         <v>46116.35019774306</v>
       </c>
       <c r="D66" s="1">
-        <v>46116.600173611114</v>
+        <v>46116.350173611114</v>
       </c>
       <c r="E66">
         <v>16742</v>
@@ -31958,7 +31958,7 @@
         <v>46116.35054157407</v>
       </c>
       <c r="D67" s="1">
-        <v>46116.60052083333</v>
+        <v>46116.35052083333</v>
       </c>
       <c r="E67">
         <v>16145</v>
@@ -32101,7 +32101,7 @@
         <v>46116.35091920139</v>
       </c>
       <c r="D68" s="1">
-        <v>46116.600856481484</v>
+        <v>46116.350856481484</v>
       </c>
       <c r="E68">
         <v>15500</v>
@@ -32244,7 +32244,7 @@
         <v>46116.3508887037</v>
       </c>
       <c r="D69" s="1">
-        <v>46116.60086805555</v>
+        <v>46116.35086805555</v>
       </c>
       <c r="E69">
         <v>15547</v>
@@ -32387,7 +32387,7 @@
         <v>46116.351260752315</v>
       </c>
       <c r="D70" s="1">
-        <v>46116.60120370371</v>
+        <v>46116.35120370371</v>
       </c>
       <c r="E70">
         <v>14915</v>
@@ -32530,7 +32530,7 @@
         <v>46116.351236284725</v>
       </c>
       <c r="D71" s="1">
-        <v>46116.60121527778</v>
+        <v>46116.35121527778</v>
       </c>
       <c r="E71">
         <v>14966</v>
@@ -32673,7 +32673,7 @@
         <v>46116.35161450232</v>
       </c>
       <c r="D72" s="1">
-        <v>46116.60155092592</v>
+        <v>46116.35155092592</v>
       </c>
       <c r="E72">
         <v>14339</v>
@@ -32816,7 +32816,7 @@
         <v>46116.351582766205</v>
       </c>
       <c r="D73" s="1">
-        <v>46116.6015625</v>
+        <v>46116.3515625</v>
       </c>
       <c r="E73">
         <v>14386</v>
@@ -32959,7 +32959,7 @@
         <v>46116.35193488426</v>
       </c>
       <c r="D74" s="1">
-        <v>46116.60189814815</v>
+        <v>46116.35189814815</v>
       </c>
       <c r="E74">
         <v>13740</v>
@@ -33102,7 +33102,7 @@
         <v>46116.35193048611</v>
       </c>
       <c r="D75" s="1">
-        <v>46116.60190972222</v>
+        <v>46116.35190972222</v>
       </c>
       <c r="E75">
         <v>13788</v>
@@ -33245,7 +33245,7 @@
         <v>46116.35230880787</v>
       </c>
       <c r="D76" s="1">
-        <v>46116.60224537037</v>
+        <v>46116.35224537037</v>
       </c>
       <c r="E76">
         <v>13166</v>
@@ -33388,7 +33388,7 @@
         <v>46116.35227768518</v>
       </c>
       <c r="D77" s="1">
-        <v>46116.60225694445</v>
+        <v>46116.35225694445</v>
       </c>
       <c r="E77">
         <v>13216</v>
@@ -33531,7 +33531,7 @@
         <v>46116.35263105324</v>
       </c>
       <c r="D78" s="1">
-        <v>46116.60260416667</v>
+        <v>46116.35260416667</v>
       </c>
       <c r="E78">
         <v>12646</v>
@@ -33674,7 +33674,7 @@
         <v>46116.353002731485</v>
       </c>
       <c r="D79" s="1">
-        <v>46116.60293981482</v>
+        <v>46116.35293981482</v>
       </c>
       <c r="E79">
         <v>12064</v>
@@ -33817,7 +33817,7 @@
         <v>46116.35297197917</v>
       </c>
       <c r="D80" s="1">
-        <v>46116.602951388886</v>
+        <v>46116.352951388886</v>
       </c>
       <c r="E80">
         <v>12092</v>
@@ -33960,7 +33960,7 @@
         <v>46116.35334421296</v>
       </c>
       <c r="D81" s="1">
-        <v>46116.60328703704</v>
+        <v>46116.35328703704</v>
       </c>
       <c r="E81">
         <v>11517</v>
@@ -34103,7 +34103,7 @@
         <v>46116.353319340276</v>
       </c>
       <c r="D82" s="1">
-        <v>46116.60329861111</v>
+        <v>46116.35329861111</v>
       </c>
       <c r="E82">
         <v>11566</v>
@@ -34246,7 +34246,7 @@
         <v>46116.353697604165</v>
       </c>
       <c r="D83" s="1">
-        <v>46116.603634259256</v>
+        <v>46116.353634259256</v>
       </c>
       <c r="E83">
         <v>10996</v>
@@ -34389,7 +34389,7 @@
         <v>46116.353676990744</v>
       </c>
       <c r="D84" s="1">
-        <v>46116.60364583333</v>
+        <v>46116.35364583333</v>
       </c>
       <c r="E84">
         <v>11044</v>
@@ -34532,7 +34532,7 @@
         <v>46116.35401681713</v>
       </c>
       <c r="D85" s="1">
-        <v>46116.60398148148</v>
+        <v>46116.35398148148</v>
       </c>
       <c r="E85">
         <v>10492</v>
@@ -34675,7 +34675,7 @@
         <v>46116.35401403935</v>
       </c>
       <c r="D86" s="1">
-        <v>46116.603993055556</v>
+        <v>46116.353993055556</v>
       </c>
       <c r="E86">
         <v>10516</v>
@@ -34818,7 +34818,7 @@
         <v>46116.35439180556</v>
       </c>
       <c r="D87" s="1">
-        <v>46116.6043287037</v>
+        <v>46116.3543287037</v>
       </c>
       <c r="E87">
         <v>9947</v>
@@ -34961,7 +34961,7 @@
         <v>46116.35437238426</v>
       </c>
       <c r="D88" s="1">
-        <v>46116.60434027778</v>
+        <v>46116.35434027778</v>
       </c>
       <c r="E88">
         <v>9996</v>
@@ -35104,7 +35104,7 @@
         <v>46116.35471530093</v>
       </c>
       <c r="D89" s="1">
-        <v>46116.6046875</v>
+        <v>46116.3546875</v>
       </c>
       <c r="E89">
         <v>9465</v>
@@ -35247,7 +35247,7 @@
         <v>46116.355063020834</v>
       </c>
       <c r="D90" s="1">
-        <v>46116.60503472222</v>
+        <v>46116.35503472222</v>
       </c>
       <c r="E90">
         <v>8960</v>
@@ -35390,7 +35390,7 @@
         <v>46116.35540512732</v>
       </c>
       <c r="D91" s="1">
-        <v>46116.60537037037</v>
+        <v>46116.35537037037</v>
       </c>
       <c r="E91">
         <v>8418</v>
@@ -35533,7 +35533,7 @@
         <v>46116.35541009259</v>
       </c>
       <c r="D92" s="1">
-        <v>46116.60538194444</v>
+        <v>46116.35538194444</v>
       </c>
       <c r="E92">
         <v>8468</v>
@@ -35676,7 +35676,7 @@
         <v>46116.35578077546</v>
       </c>
       <c r="D93" s="1">
-        <v>46116.605717592596</v>
+        <v>46116.355717592596</v>
       </c>
       <c r="E93">
         <v>7921</v>
@@ -35819,7 +35819,7 @@
         <v>46116.355758032405</v>
       </c>
       <c r="D94" s="1">
-        <v>46116.605729166666</v>
+        <v>46116.355729166666</v>
       </c>
       <c r="E94">
         <v>7970</v>
@@ -35962,7 +35962,7 @@
         <v>46116.356105405095</v>
       </c>
       <c r="D95" s="1">
-        <v>46116.60606481481</v>
+        <v>46116.35606481481</v>
       </c>
       <c r="E95">
         <v>7410</v>
@@ -36105,7 +36105,7 @@
         <v>46116.35610469907</v>
       </c>
       <c r="D96" s="1">
-        <v>46116.60607638889</v>
+        <v>46116.35607638889</v>
       </c>
       <c r="E96">
         <v>7455</v>
@@ -36248,7 +36248,7 @@
         <v>46116.35647543982</v>
       </c>
       <c r="D97" s="1">
-        <v>46116.606412037036</v>
+        <v>46116.356412037036</v>
       </c>
       <c r="E97">
         <v>6875</v>
@@ -36391,7 +36391,7 @@
         <v>46116.35645241898</v>
       </c>
       <c r="D98" s="1">
-        <v>46116.60642361111</v>
+        <v>46116.35642361111</v>
       </c>
       <c r="E98">
         <v>6921</v>
@@ -36534,7 +36534,7 @@
         <v>46116.35678857639</v>
       </c>
       <c r="D99" s="1">
-        <v>46116.60675925926</v>
+        <v>46116.35675925926</v>
       </c>
       <c r="E99">
         <v>6301</v>
@@ -36677,7 +36677,7 @@
         <v>46116.356800636575</v>
       </c>
       <c r="D100" s="1">
-        <v>46116.606770833336</v>
+        <v>46116.356770833336</v>
       </c>
       <c r="E100">
         <v>6343</v>
@@ -36820,7 +36820,7 @@
         <v>46116.35717038195</v>
       </c>
       <c r="D101" s="1">
-        <v>46116.60710648148</v>
+        <v>46116.35710648148</v>
       </c>
       <c r="E101">
         <v>5749</v>
@@ -36963,7 +36963,7 @@
         <v>46116.35714704861</v>
       </c>
       <c r="D102" s="1">
-        <v>46116.60711805556</v>
+        <v>46116.35711805556</v>
       </c>
       <c r="E102">
         <v>5794</v>

</xml_diff>